<commit_message>
Disclose the XLC splice inside the workbook
The deck discloses the splice on the chart and the README states it, but
the workbook did not. Anyone reading only the Excel would see Alphabet's
sector benchmark returning 48.1% with no indication that the series is
XLK before June 2018, and would get a different figure checking XLC alone.

Adds a sector-benchmark line to the Read me and a footnote to both sheets
that use the spliced series. Also drops the redundant ticker from
Schlumberger's company name, which has its own column.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019d1fAgUUAUCwhg9kM6iuzh
</commit_message>
<xml_diff>
--- a/finc13303-portfolio-performance/deliverables/FINC13303_Ass2_PerformanceWorkbook_14053836_OConnor.xlsx
+++ b/finc13303-portfolio-performance/deliverables/FINC13303_Ass2_PerformanceWorkbook_14053836_OConnor.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -739,146 +739,158 @@
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>Sector benchmarks</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>The eleven SPDR GICS sector ETFs. XLC launched June 2018, so XLK stands in for Communication Services before that date</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
           <t>Excluded</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Transaction costs, market impact, taxes, cash drag</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="7" t="inlineStr"/>
-      <c r="B20" s="8" t="inlineStr"/>
-    </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Contents</t>
-        </is>
-      </c>
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Holdings</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Target weights, tiers, and per-holding six-year statistics</t>
+          <t>Contents</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Performance summary</t>
+          <t>Holdings</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Full metric table for the fund, the variants and the benchmarks</t>
+          <t>Target weights, tiers, and per-holding six-year statistics</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Annual returns</t>
+          <t>Performance summary</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Calendar-year returns for every series</t>
+          <t>Full metric table for the fund, the variants and the benchmarks</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Regressions</t>
+          <t>Annual returns</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>CAPM, FF3, FF5 and FF5+momentum output</t>
+          <t>Calendar-year returns for every series</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Attribution</t>
+          <t>Regressions</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Brinson–Fachler decomposition and per-holding contribution</t>
+          <t>CAPM, FF3, FF5 and FF5+momentum output</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Seasonality</t>
+          <t>Attribution</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Monthly return grid by year and calendar-month averages</t>
+          <t>Brinson–Fachler decomposition and per-holding contribution</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Monthly returns</t>
+          <t>Seasonality</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>The 72-month return series for every strategy and benchmark</t>
+          <t>Monthly return grid by year and calendar-month averages</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Stock returns</t>
+          <t>Monthly returns</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>The 72-month return series for the eleven holdings</t>
+          <t>The 72-month return series for every strategy and benchmark</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Weight path</t>
+          <t>Stock returns</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Portfolio weights at the start of each month, as run</t>
+          <t>The 72-month return series for the eleven holdings</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
+          <t>Weight path</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Portfolio weights at the start of each month, as run</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
           <t>Factor data</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Fama–French factors and the risk-free rate, as used</t>
         </is>
@@ -5975,7 +5987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6772,7 +6784,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Schlumberger (SLB)</t>
+          <t>Schlumberger</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -6900,6 +6912,13 @@
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Contribution is the compounded contribution of each holding to the fund's 179.2% cumulative return, using the realised weight path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>XLC, the Communication Services sector ETF, launched in June 2018. The Communication Services sleeve is spliced with XLK before that date, so the Alphabet sector comparison and the Brinson attribution both cover the full 72 months.</t>
         </is>
       </c>
     </row>
@@ -9161,7 +9180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9488,7 +9507,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Schlumberger (SLB)</t>
+          <t>Schlumberger</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
@@ -9598,6 +9617,13 @@
       </c>
       <c r="F29" s="9" t="n">
         <v>1.179740561049385</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>XLC, the Communication Services sector ETF, launched in June 2018. The Communication Services sleeve is spliced with XLK before that date, so the Alphabet sector comparison and the Brinson attribution both cover the full 72 months.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>